<commit_message>
Add artwork assets for La Haine and Mirror
</commit_message>
<xml_diff>
--- a/outputs/catalog/Movie Collection Catalog.xlsx
+++ b/outputs/catalog/Movie Collection Catalog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rafd8d1fd9d7f47b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="2" r:id="R5c69db1816234386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="3" r:id="Raffd5ea9e70a463e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R9018527467564d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="2" r:id="R2d6af7b75a2c4ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookups" sheetId="3" r:id="Re74978836af74e94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13693,10 +13693,18 @@
       <x:c r="AH165" t="str">
         <x:v>After a chaotic night of rioting in a marginal suburb of Paris, three young friends, Vinz, Hubert and Saïd, wander around unoccupied waiting for news about the state of health of a mutual friend who has been seriously injured when confronting the police.</x:v>
       </x:c>
-      <x:c r="AI165" t="str"/>
-      <x:c r="AJ165" t="str"/>
-      <x:c r="AK165" t="str"/>
-      <x:c r="AL165" t="str"/>
+      <x:c r="AI165" t="str">
+        <x:v>./posters/movie-164-back.jpg</x:v>
+      </x:c>
+      <x:c r="AJ165" t="str">
+        <x:v>./posters/movie-164-spine.png</x:v>
+      </x:c>
+      <x:c r="AK165" t="str">
+        <x:v>TMDb</x:v>
+      </x:c>
+      <x:c r="AL165" t="str">
+        <x:v>https://www.themoviedb.org/movie/406</x:v>
+      </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="7" t="str">
@@ -13861,10 +13869,18 @@
       <x:c r="AH167" t="str">
         <x:v>A dying man in his forties recalls his childhood, his mother, the war and personal moments that tell of and juxtapose pivotal moments in Soviet history with daily life.</x:v>
       </x:c>
-      <x:c r="AI167" t="str"/>
-      <x:c r="AJ167" t="str"/>
-      <x:c r="AK167" t="str"/>
-      <x:c r="AL167" t="str"/>
+      <x:c r="AI167" t="str">
+        <x:v>./posters/movie-166-back.jpg</x:v>
+      </x:c>
+      <x:c r="AJ167" t="str">
+        <x:v>./posters/movie-166-spine.png</x:v>
+      </x:c>
+      <x:c r="AK167" t="str">
+        <x:v>TMDb</x:v>
+      </x:c>
+      <x:c r="AL167" t="str">
+        <x:v>https://www.themoviedb.org/movie/1396</x:v>
+      </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="7" t="str">
@@ -22803,7 +22819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdebeb81547794695"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13bf40d513934129"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>